<commit_message>
Add Category search, case-insensitive duplicate and count testcases
- No-results search shows empty state message
- Clearing search restores full list; count matches fresh list API
- Duplicate name check is case-insensitive (lower/UPPER)
- Header count -1 after each delete; returns to initial count after cleanup
- Drop unused exports from Categories page object
- Update test plan notes for CAT-008/022/023/049/105

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Category_Module_Test_Plan_and_TestCases.xlsx
+++ b/Category_Module_Test_Plan_and_TestCases.xlsx
@@ -1676,7 +1676,11 @@
       </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Automated: 'Verify Categories page UI elements are displayed', 'Clearing search restores the full list matching API count', 'Category count returns to initial and matches API after deletes'</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2413,7 +2417,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>No rows; friendly 'no categories found' message</t>
+          <t>No rows; message 'No categories match "&lt;text&gt;"' shown</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -2423,7 +2427,11 @@
       </c>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Automated: 'Search with no matching category shows empty state'</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2464,7 +2472,7 @@
       <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Full list and original count restored</t>
+          <t>Full list restored; rows == header count; header count stays at store total even while searching</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2474,7 +2482,11 @@
       </c>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>Automated: 'Clearing search restores the full list matching API count'</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3845,7 +3857,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Duplicate error (case-insensitive) as per business rule</t>
+          <t>Duplicate check is case-insensitive: lowercase/UPPERCASE of an existing name fails with 'The name is Already exist' (API status Failed)</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -3855,7 +3867,11 @@
       </c>
       <c r="K50" s="2" t="inlineStr"/>
       <c r="L50" s="2" t="inlineStr"/>
-      <c r="M50" s="2" t="inlineStr"/>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>Automated: 'Verify duplicate check is case-insensitive'</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -6836,7 +6852,11 @@
       </c>
       <c r="K106" s="2" t="inlineStr"/>
       <c r="L106" s="2" t="inlineStr"/>
-      <c r="M106" s="2" t="inlineStr"/>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>Automated: 'Verify Delete category' (header count -1 checked per delete)</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">

</xml_diff>